<commit_message>
Finish creating test data - 16.04.2025
</commit_message>
<xml_diff>
--- a/1. Database Design/Java23 LuuNgocYenNhu Database Design.xlsx
+++ b/1. Database Design/Java23 LuuNgocYenNhu Database Design.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java23\3. Database\1. Database Design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\java23\3. Database\1. Database Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{046FDCEA-E48F-47C1-A4C0-9185C522C388}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C7F5D9A-2C5F-403D-84D9-426C824A384D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="588" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="588" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="B1. Mô hình quan niệm" sheetId="1" r:id="rId1"/>
@@ -18,23 +18,13 @@
     <sheet name="B2. ERD - Mô hình logic" sheetId="2" r:id="rId3"/>
     <sheet name="B3. Mô hình quan hệ" sheetId="6" r:id="rId4"/>
     <sheet name="B4. Mô hình vật lý" sheetId="4" r:id="rId5"/>
-    <sheet name="RD - Mô hình quan hệ" sheetId="3" r:id="rId6"/>
+    <sheet name="B5. Tạo dữ liệu mẫu" sheetId="7" r:id="rId6"/>
+    <sheet name="RD - Mô hình quan hệ" sheetId="3" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -227,18 +217,35 @@
   <commentList>
     <comment ref="K6" authorId="0" shapeId="0" xr:uid="{D2762586-1568-4CA1-84B1-25C4A6B7BF3D}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Khách
 Nhân Viên
 Quản Lý 
 Giám Đốc</t>
+        </r>
       </text>
     </comment>
     <comment ref="L6" authorId="1" shapeId="0" xr:uid="{5BB71AC4-9659-4B49-AE00-20328F749FE8}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Chờ xử lý
@@ -248,41 +255,78 @@
 Giao hàng thành công
 Giao hàng thất bại
 Hủy đơn hàng</t>
+        </r>
       </text>
     </comment>
     <comment ref="N6" authorId="2" shapeId="0" xr:uid="{B0B8351A-F8B3-4EDE-8A43-27DE73070A70}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Thanh toán khi nhận hàng
 Thanh toán online - chuyển khoản
 Thanh toán online - thẻ ghi nợ
 </t>
+        </r>
       </text>
     </comment>
     <comment ref="Q7" authorId="3" shapeId="0" xr:uid="{F97C4A89-C3BD-42B8-81A3-F88B0C7B2B49}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Số lượng bán của mặt hàng trong đơn hàng</t>
+        </r>
       </text>
     </comment>
     <comment ref="D10" authorId="4" shapeId="0" xr:uid="{6B85BF31-59E0-4C41-93B2-A52F1794EB43}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Số lượng tồn kho theo mặt hàng, kích cỡ</t>
+        </r>
       </text>
     </comment>
     <comment ref="G12" authorId="5" shapeId="0" xr:uid="{757E2222-AC3E-4A43-98F1-5381EF486FA8}">
       <text>
-        <t>[Threaded comment]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Người tạo</t>
+        </r>
       </text>
     </comment>
   </commentList>
@@ -290,7 +334,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1045" uniqueCount="496">
   <si>
     <t>MatHang</t>
   </si>
@@ -1850,12 +1894,105 @@
   <si>
     <t>file://img04</t>
   </si>
+  <si>
+    <t>Áo</t>
+  </si>
+  <si>
+    <t>Quần</t>
+  </si>
+  <si>
+    <t>Giày</t>
+  </si>
+  <si>
+    <t>Dép</t>
+  </si>
+  <si>
+    <t>Mũ</t>
+  </si>
+  <si>
+    <t>Thắt lưng</t>
+  </si>
+  <si>
+    <t>Túi xách</t>
+  </si>
+  <si>
+    <t>Áo 1</t>
+  </si>
+  <si>
+    <t>Áo 2</t>
+  </si>
+  <si>
+    <t>Áo 3</t>
+  </si>
+  <si>
+    <t>Quần 4</t>
+  </si>
+  <si>
+    <t>Quần 5</t>
+  </si>
+  <si>
+    <t>Giày 6</t>
+  </si>
+  <si>
+    <t>Giày 7</t>
+  </si>
+  <si>
+    <t>Giày 8</t>
+  </si>
+  <si>
+    <t>Giày 9</t>
+  </si>
+  <si>
+    <t>Giày 10</t>
+  </si>
+  <si>
+    <t>Giép 11</t>
+  </si>
+  <si>
+    <t>Áo 12</t>
+  </si>
+  <si>
+    <t>Giép 13</t>
+  </si>
+  <si>
+    <t>Mũ 14</t>
+  </si>
+  <si>
+    <t>Mũ 15</t>
+  </si>
+  <si>
+    <t>Thắt lưng 16</t>
+  </si>
+  <si>
+    <t>Thắt lưng 17</t>
+  </si>
+  <si>
+    <t>Mũ 18</t>
+  </si>
+  <si>
+    <t>Túi xách 1</t>
+  </si>
+  <si>
+    <t>Túi xách 2</t>
+  </si>
+  <si>
+    <t>C01_REF_ITEM_ID</t>
+  </si>
+  <si>
+    <t>T04_ITEMGROUP</t>
+  </si>
+  <si>
+    <t>C04_ITEMGROUP_ID</t>
+  </si>
+  <si>
+    <t>C04_ITEMGROUP_NAME</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2003,6 +2140,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFC000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -2120,7 +2280,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2297,6 +2457,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2317,7 +2483,16 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2643,21 +2818,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A4:L24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="8" width="16.85546875" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" customWidth="1"/>
+    <col min="5" max="8" width="16.88671875" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" customWidth="1"/>
+    <col min="10" max="10" width="18.6640625" customWidth="1"/>
     <col min="11" max="11" width="21" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" customWidth="1"/>
-    <col min="13" max="18" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="17.44140625" customWidth="1"/>
+    <col min="13" max="18" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -2692,7 +2867,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -2727,7 +2902,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="50" t="s">
         <v>253</v>
       </c>
@@ -2762,7 +2937,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>254</v>
       </c>
@@ -2792,7 +2967,7 @@
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
     </row>
-    <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>255</v>
       </c>
@@ -2822,7 +2997,7 @@
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
     </row>
-    <row r="9" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="50" t="s">
         <v>225</v>
       </c>
@@ -2845,7 +3020,7 @@
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
     </row>
-    <row r="10" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="50" t="s">
         <v>252</v>
       </c>
@@ -2868,7 +3043,7 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="50" t="s">
         <v>251</v>
       </c>
@@ -2891,7 +3066,7 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="50" t="s">
         <v>250</v>
       </c>
@@ -2908,7 +3083,7 @@
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="2" t="s">
         <v>17</v>
       </c>
@@ -2922,7 +3097,7 @@
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
     </row>
-    <row r="14" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -2935,7 +3110,7 @@
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
     </row>
-    <row r="15" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -2948,7 +3123,7 @@
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
     </row>
-    <row r="16" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -2961,7 +3136,7 @@
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -2974,7 +3149,7 @@
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
     </row>
-    <row r="18" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -2987,7 +3162,7 @@
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
     </row>
-    <row r="19" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -3000,7 +3175,7 @@
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
     </row>
-    <row r="20" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -3013,12 +3188,12 @@
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="15" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="24" spans="2:12" s="15" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="2:12" s="15" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3029,27 +3204,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00967ACB-CFA1-460B-A734-E9F64BF353E8}">
   <dimension ref="A2:P58"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="9" width="16.85546875" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="13" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="9" width="16.88671875" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" customWidth="1"/>
+    <col min="11" max="13" width="18.6640625" customWidth="1"/>
     <col min="14" max="14" width="21" customWidth="1"/>
-    <col min="15" max="15" width="17.42578125" customWidth="1"/>
-    <col min="16" max="16" width="18.28515625" customWidth="1"/>
-    <col min="17" max="21" width="12.7109375" customWidth="1"/>
+    <col min="15" max="15" width="17.44140625" customWidth="1"/>
+    <col min="16" max="16" width="18.33203125" customWidth="1"/>
+    <col min="17" max="21" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="F2" s="15" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -3093,7 +3268,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="52" t="s">
         <v>1</v>
       </c>
@@ -3137,7 +3312,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="50" t="s">
         <v>253</v>
       </c>
@@ -3181,7 +3356,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>254</v>
       </c>
@@ -3220,7 +3395,7 @@
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>255</v>
       </c>
@@ -3253,7 +3428,7 @@
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="50" t="s">
         <v>252</v>
       </c>
@@ -3279,7 +3454,7 @@
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
     </row>
-    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="50" t="s">
         <v>251</v>
       </c>
@@ -3303,7 +3478,7 @@
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
     </row>
-    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="50" t="s">
         <v>250</v>
       </c>
@@ -3327,7 +3502,7 @@
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="2" t="s">
         <v>17</v>
       </c>
@@ -3347,7 +3522,7 @@
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
     </row>
-    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -3362,7 +3537,7 @@
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
     </row>
-    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -3378,7 +3553,7 @@
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
     </row>
-    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -3394,7 +3569,7 @@
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
     </row>
-    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -3410,7 +3585,7 @@
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
     </row>
-    <row r="17" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -3426,7 +3601,7 @@
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
     </row>
-    <row r="18" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -3442,7 +3617,7 @@
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
     </row>
-    <row r="19" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -3458,7 +3633,7 @@
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
     </row>
-    <row r="20" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -3474,12 +3649,12 @@
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>70</v>
       </c>
@@ -3493,7 +3668,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="24" spans="2:16" s="15" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:16" s="15" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24"/>
       <c r="C24" t="s">
         <v>71</v>
@@ -3519,7 +3694,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B25" s="9" t="s">
         <v>72</v>
       </c>
@@ -3548,7 +3723,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B26" s="9" t="s">
         <v>73</v>
       </c>
@@ -3575,7 +3750,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C27" t="s">
         <v>74</v>
       </c>
@@ -3599,7 +3774,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
       <c r="H28" s="44" t="s">
         <v>274</v>
       </c>
@@ -3616,7 +3791,7 @@
       <c r="O28" s="44"/>
       <c r="P28" s="44"/>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
       <c r="H29" s="44" t="s">
         <v>274</v>
       </c>
@@ -3633,7 +3808,7 @@
       <c r="O29" s="44"/>
       <c r="P29" s="44"/>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
       <c r="G30" s="53" t="s">
         <v>276</v>
       </c>
@@ -3653,14 +3828,14 @@
       <c r="O30" s="44"/>
       <c r="P30" s="44"/>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
       <c r="N31" s="44" t="s">
         <v>236</v>
       </c>
       <c r="O31" s="44"/>
       <c r="P31" s="44"/>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
       <c r="N32" s="5" t="s">
         <v>237</v>
       </c>
@@ -3668,7 +3843,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
       <c r="N33" s="5">
         <v>1</v>
       </c>
@@ -3676,7 +3851,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
       <c r="H34" t="s">
         <v>0</v>
       </c>
@@ -3687,7 +3862,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
       <c r="H35" s="50" t="s">
         <v>1</v>
       </c>
@@ -3704,7 +3879,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
       <c r="H36" s="44" t="s">
         <v>267</v>
       </c>
@@ -3721,7 +3896,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
       <c r="H37" s="44" t="s">
         <v>268</v>
       </c>
@@ -3732,7 +3907,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:15" x14ac:dyDescent="0.3">
       <c r="H38" s="44" t="s">
         <v>269</v>
       </c>
@@ -3746,7 +3921,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B39" s="44"/>
       <c r="C39" s="44"/>
       <c r="D39" s="44"/>
@@ -3758,7 +3933,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B40" s="44"/>
       <c r="C40" s="44"/>
       <c r="D40" s="44"/>
@@ -3770,7 +3945,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B41" s="44"/>
       <c r="C41" s="44"/>
       <c r="D41" s="44"/>
@@ -3782,7 +3957,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="42" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B42" s="44"/>
       <c r="C42" s="44"/>
       <c r="D42" s="44"/>
@@ -3794,7 +3969,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="43" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B43" s="1" t="s">
         <v>295</v>
       </c>
@@ -3808,7 +3983,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="44" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B44" s="2" t="s">
         <v>239</v>
       </c>
@@ -3829,7 +4004,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="45" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B45" s="44" t="s">
         <v>294</v>
       </c>
@@ -3850,7 +4025,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="46" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B46" s="44" t="s">
         <v>294</v>
       </c>
@@ -3871,7 +4046,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="47" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B47" s="44" t="s">
         <v>294</v>
       </c>
@@ -3889,7 +4064,7 @@
       </c>
       <c r="G47" s="44"/>
     </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B48" s="44"/>
       <c r="C48" s="44"/>
       <c r="D48" s="44"/>
@@ -3898,7 +4073,7 @@
       <c r="G48" s="44"/>
       <c r="H48" s="44"/>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B49" s="44"/>
       <c r="C49" s="44"/>
       <c r="D49" s="44"/>
@@ -3907,7 +4082,7 @@
       <c r="G49" s="44"/>
       <c r="H49" s="44"/>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B50" s="44" t="s">
         <v>262</v>
       </c>
@@ -3918,7 +4093,7 @@
       <c r="G50" s="44"/>
       <c r="H50" s="44"/>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B51" s="2" t="s">
         <v>239</v>
       </c>
@@ -3933,7 +4108,7 @@
       <c r="G51" s="44"/>
       <c r="H51" s="44"/>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B52" s="44" t="s">
         <v>294</v>
       </c>
@@ -3948,7 +4123,7 @@
       <c r="G52" s="44"/>
       <c r="H52" s="44"/>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B53" s="44" t="s">
         <v>296</v>
       </c>
@@ -3963,7 +4138,7 @@
       <c r="G53" s="44"/>
       <c r="H53" s="44"/>
     </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B54" s="44" t="s">
         <v>297</v>
       </c>
@@ -3978,7 +4153,7 @@
       <c r="G54" s="44"/>
       <c r="H54" s="44"/>
     </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B55" s="44"/>
       <c r="C55" s="44"/>
       <c r="D55" s="44"/>
@@ -3987,7 +4162,7 @@
       <c r="G55" s="44"/>
       <c r="H55" s="44"/>
     </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B56" s="44"/>
       <c r="C56" s="44"/>
       <c r="D56" s="44"/>
@@ -3996,7 +4171,7 @@
       <c r="G56" s="44"/>
       <c r="H56" s="44"/>
     </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B57" s="44"/>
       <c r="C57" s="44"/>
       <c r="D57" s="44"/>
@@ -4005,7 +4180,7 @@
       <c r="G57" s="44"/>
       <c r="H57" s="44"/>
     </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B58" s="44"/>
       <c r="C58" s="44"/>
       <c r="D58" s="44"/>
@@ -4024,16 +4199,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:U43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" customWidth="1"/>
-    <col min="9" max="9" width="10.42578125" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" customWidth="1"/>
-    <col min="16" max="16" width="11.85546875" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" customWidth="1"/>
+    <col min="9" max="9" width="10.44140625" customWidth="1"/>
+    <col min="15" max="15" width="12.5546875" customWidth="1"/>
+    <col min="16" max="16" width="11.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>107</v>
       </c>
@@ -4046,7 +4221,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -4054,7 +4229,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -4063,10 +4238,10 @@
       </c>
       <c r="P4" s="47"/>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="N5" s="47"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B7" s="10" t="s">
         <v>43</v>
       </c>
@@ -4078,7 +4253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="D8" s="5"/>
       <c r="P8" s="21" t="s">
         <v>59</v>
@@ -4087,7 +4262,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
         <v>28</v>
       </c>
@@ -4128,7 +4303,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
         <v>45</v>
       </c>
@@ -4169,7 +4344,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B11" s="4" t="s">
         <v>63</v>
       </c>
@@ -4204,7 +4379,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B12" s="4" t="s">
         <v>46</v>
       </c>
@@ -4239,7 +4414,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="4" t="s">
         <v>57</v>
       </c>
@@ -4255,14 +4430,14 @@
       <c r="Q13" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="R13" s="69" t="s">
+      <c r="R13" s="71" t="s">
         <v>68</v>
       </c>
-      <c r="S13" s="69"/>
-      <c r="T13" s="69"/>
-      <c r="U13" s="69"/>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="S13" s="71"/>
+      <c r="T13" s="71"/>
+      <c r="U13" s="71"/>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="D14" s="5"/>
       <c r="O14" s="13" t="s">
         <v>43</v>
@@ -4273,20 +4448,20 @@
       <c r="Q14" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="R14" s="69"/>
-      <c r="S14" s="69"/>
-      <c r="T14" s="69"/>
-      <c r="U14" s="69"/>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="R14" s="71"/>
+      <c r="S14" s="71"/>
+      <c r="T14" s="71"/>
+      <c r="U14" s="71"/>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="J16" s="47"/>
     </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B17" s="11" t="s">
         <v>37</v>
       </c>
@@ -4306,7 +4481,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" x14ac:dyDescent="0.3">
       <c r="G18" s="5"/>
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
@@ -4317,7 +4492,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B19" s="6" t="s">
         <v>38</v>
       </c>
@@ -4346,7 +4521,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B20" s="12">
         <v>1</v>
       </c>
@@ -4369,7 +4544,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B21" s="4" t="s">
         <v>54</v>
       </c>
@@ -4401,7 +4576,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B22" s="4">
         <v>3</v>
       </c>
@@ -4428,7 +4603,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:20" x14ac:dyDescent="0.3">
       <c r="G23" s="5">
         <v>4</v>
       </c>
@@ -4445,7 +4620,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:20" x14ac:dyDescent="0.3">
       <c r="G24" s="5">
         <v>5</v>
       </c>
@@ -4459,7 +4634,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:20" x14ac:dyDescent="0.3">
       <c r="G25" s="5">
         <v>6</v>
       </c>
@@ -4473,7 +4648,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:20" x14ac:dyDescent="0.3">
       <c r="G26" s="5">
         <v>7</v>
       </c>
@@ -4490,7 +4665,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:20" x14ac:dyDescent="0.3">
       <c r="N27" s="47" t="s">
         <v>1</v>
       </c>
@@ -4498,7 +4673,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>69</v>
       </c>
@@ -4509,7 +4684,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
         <v>70</v>
       </c>
@@ -4520,7 +4695,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="30" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:20" x14ac:dyDescent="0.3">
       <c r="C30" t="s">
         <v>71</v>
       </c>
@@ -4531,7 +4706,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="31" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B31" s="9" t="s">
         <v>72</v>
       </c>
@@ -4546,7 +4721,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="32" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B32" s="9" t="s">
         <v>73</v>
       </c>
@@ -4564,7 +4739,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
       <c r="C33" t="s">
         <v>74</v>
       </c>
@@ -4575,7 +4750,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
       <c r="N34">
         <v>3</v>
       </c>
@@ -4583,7 +4758,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>304</v>
       </c>
@@ -4595,7 +4770,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>305</v>
       </c>
@@ -4603,31 +4778,31 @@
       <c r="I36" s="44"/>
       <c r="J36" s="44"/>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
       <c r="I37" s="44"/>
       <c r="J37" s="44"/>
     </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:15" x14ac:dyDescent="0.3">
       <c r="I38" s="44"/>
       <c r="J38" s="44"/>
     </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
       <c r="I39" s="44"/>
       <c r="J39" s="44"/>
     </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
       <c r="I40" s="44"/>
       <c r="J40" s="44"/>
     </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:15" x14ac:dyDescent="0.3">
       <c r="I41" s="44"/>
       <c r="J41" s="44"/>
     </row>
-    <row r="42" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:15" x14ac:dyDescent="0.3">
       <c r="I42" s="48"/>
       <c r="J42" s="48"/>
     </row>
-    <row r="43" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:15" x14ac:dyDescent="0.3">
       <c r="I43" s="44"/>
       <c r="J43" s="44"/>
     </row>
@@ -4643,27 +4818,27 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AD2C7DF-5616-418E-B427-D50946AF144B}">
   <dimension ref="A2:Q58"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="9" width="16.85546875" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="13" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="9" width="16.88671875" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" customWidth="1"/>
+    <col min="11" max="13" width="18.6640625" customWidth="1"/>
     <col min="14" max="14" width="21" customWidth="1"/>
-    <col min="15" max="15" width="17.42578125" customWidth="1"/>
-    <col min="16" max="16" width="18.28515625" customWidth="1"/>
-    <col min="17" max="21" width="12.7109375" customWidth="1"/>
+    <col min="15" max="15" width="17.44140625" customWidth="1"/>
+    <col min="16" max="16" width="18.33203125" customWidth="1"/>
+    <col min="17" max="21" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="F2" s="15" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="3" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>276</v>
       </c>
@@ -4704,7 +4879,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -4748,7 +4923,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="52" t="s">
         <v>1</v>
       </c>
@@ -4792,7 +4967,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="50" t="s">
         <v>253</v>
       </c>
@@ -4836,7 +5011,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>254</v>
       </c>
@@ -4875,7 +5050,7 @@
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>255</v>
       </c>
@@ -4908,7 +5083,7 @@
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="50" t="s">
         <v>252</v>
       </c>
@@ -4934,7 +5109,7 @@
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
     </row>
-    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="50" t="s">
         <v>251</v>
       </c>
@@ -4958,7 +5133,7 @@
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
     </row>
-    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="50" t="s">
         <v>250</v>
       </c>
@@ -4982,7 +5157,7 @@
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="2" t="s">
         <v>17</v>
       </c>
@@ -5002,7 +5177,7 @@
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
     </row>
-    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -5017,7 +5192,7 @@
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
     </row>
-    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -5033,7 +5208,7 @@
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
     </row>
-    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -5049,7 +5224,7 @@
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
     </row>
-    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -5065,7 +5240,7 @@
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
     </row>
-    <row r="17" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -5081,7 +5256,7 @@
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
     </row>
-    <row r="18" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -5097,7 +5272,7 @@
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
     </row>
-    <row r="19" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -5113,7 +5288,7 @@
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
     </row>
-    <row r="20" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -5129,12 +5304,12 @@
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
     </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:17" x14ac:dyDescent="0.3">
       <c r="C23" s="54" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="24" spans="2:17" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:17" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24"/>
       <c r="C24" s="20" t="s">
         <v>307</v>
@@ -5153,17 +5328,17 @@
       <c r="P24"/>
       <c r="Q24"/>
     </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:17" x14ac:dyDescent="0.3">
       <c r="C25" s="20" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:17" x14ac:dyDescent="0.3">
       <c r="C27" s="54" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:17" x14ac:dyDescent="0.3">
       <c r="C28" s="20" t="s">
         <v>310</v>
       </c>
@@ -5173,7 +5348,7 @@
       <c r="O28" s="44"/>
       <c r="P28" s="44"/>
     </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:17" x14ac:dyDescent="0.3">
       <c r="C29" s="20" t="s">
         <v>311</v>
       </c>
@@ -5183,47 +5358,47 @@
       <c r="O29" s="44"/>
       <c r="P29" s="44"/>
     </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:17" x14ac:dyDescent="0.3">
       <c r="L30" s="44"/>
       <c r="M30" s="44"/>
       <c r="N30" s="44"/>
       <c r="O30" s="44"/>
       <c r="P30" s="44"/>
     </row>
-    <row r="31" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:17" x14ac:dyDescent="0.3">
       <c r="C31" s="54" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:17" x14ac:dyDescent="0.3">
       <c r="C32" s="20" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
       <c r="C33" s="20" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
       <c r="C35" s="54" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
       <c r="C36" s="20" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
       <c r="C37" s="20"/>
     </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:8" x14ac:dyDescent="0.3">
       <c r="C38" s="20" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B39" s="44"/>
       <c r="C39" s="56" t="s">
         <v>326</v>
@@ -5234,23 +5409,23 @@
       <c r="G39" s="44"/>
       <c r="H39" s="44"/>
     </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:8" x14ac:dyDescent="0.3">
       <c r="G40" s="44"/>
       <c r="H40" s="44"/>
     </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:8" x14ac:dyDescent="0.3">
       <c r="G41" s="44"/>
       <c r="H41" s="44"/>
     </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:8" x14ac:dyDescent="0.3">
       <c r="G42" s="44"/>
       <c r="H42" s="44"/>
     </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:8" x14ac:dyDescent="0.3">
       <c r="G43" s="44"/>
       <c r="H43" s="44"/>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B49" s="44"/>
       <c r="C49" s="44"/>
       <c r="D49" s="44"/>
@@ -5259,32 +5434,32 @@
       <c r="G49" s="44"/>
       <c r="H49" s="44"/>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
       <c r="F50" s="44"/>
       <c r="G50" s="44"/>
       <c r="H50" s="44"/>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
       <c r="F51" s="44"/>
       <c r="G51" s="44"/>
       <c r="H51" s="44"/>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
       <c r="F52" s="44"/>
       <c r="G52" s="44"/>
       <c r="H52" s="44"/>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
       <c r="F53" s="44"/>
       <c r="G53" s="44"/>
       <c r="H53" s="44"/>
     </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
       <c r="F54" s="44"/>
       <c r="G54" s="44"/>
       <c r="H54" s="44"/>
     </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B55" s="44"/>
       <c r="C55" s="44"/>
       <c r="D55" s="44"/>
@@ -5293,7 +5468,7 @@
       <c r="G55" s="44"/>
       <c r="H55" s="44"/>
     </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B56" s="44"/>
       <c r="C56" s="44"/>
       <c r="D56" s="44"/>
@@ -5302,7 +5477,7 @@
       <c r="G56" s="44"/>
       <c r="H56" s="44"/>
     </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B57" s="44"/>
       <c r="C57" s="44"/>
       <c r="D57" s="44"/>
@@ -5311,7 +5486,7 @@
       <c r="G57" s="44"/>
       <c r="H57" s="44"/>
     </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B58" s="44"/>
       <c r="C58" s="44"/>
       <c r="D58" s="44"/>
@@ -5330,37 +5505,37 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:T58"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" customWidth="1"/>
+    <col min="4" max="4" width="20.44140625" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="21.140625" customWidth="1"/>
-    <col min="7" max="7" width="29.85546875" customWidth="1"/>
-    <col min="8" max="8" width="24.85546875" customWidth="1"/>
-    <col min="9" max="9" width="21.85546875" customWidth="1"/>
-    <col min="10" max="10" width="21.7109375" customWidth="1"/>
-    <col min="11" max="11" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="21.109375" customWidth="1"/>
+    <col min="7" max="7" width="29.88671875" customWidth="1"/>
+    <col min="8" max="8" width="24.88671875" customWidth="1"/>
+    <col min="9" max="9" width="21.88671875" customWidth="1"/>
+    <col min="10" max="10" width="21.6640625" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" customWidth="1"/>
     <col min="12" max="12" width="26" customWidth="1"/>
-    <col min="13" max="13" width="27.7109375" customWidth="1"/>
-    <col min="14" max="14" width="30.85546875" customWidth="1"/>
-    <col min="15" max="17" width="22.7109375" customWidth="1"/>
-    <col min="18" max="18" width="24.140625" customWidth="1"/>
-    <col min="19" max="19" width="35.140625" customWidth="1"/>
-    <col min="20" max="20" width="21.5703125" customWidth="1"/>
-    <col min="21" max="22" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="27.6640625" customWidth="1"/>
+    <col min="14" max="14" width="30.88671875" customWidth="1"/>
+    <col min="15" max="17" width="22.6640625" customWidth="1"/>
+    <col min="18" max="18" width="24.109375" customWidth="1"/>
+    <col min="19" max="19" width="35.109375" customWidth="1"/>
+    <col min="20" max="20" width="21.5546875" customWidth="1"/>
+    <col min="21" max="22" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>331</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
     </row>
-    <row r="3" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:20" x14ac:dyDescent="0.3">
       <c r="D3" s="5" t="s">
         <v>349</v>
       </c>
@@ -5368,7 +5543,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="4" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>332</v>
       </c>
@@ -5427,7 +5602,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="5" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="59" t="s">
         <v>333</v>
       </c>
@@ -5486,14 +5661,14 @@
         <v>440</v>
       </c>
     </row>
-    <row r="6" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="2" t="s">
         <v>334</v>
       </c>
       <c r="C6" s="60" t="s">
         <v>341</v>
       </c>
-      <c r="D6" s="76" t="s">
+      <c r="D6" s="70" t="s">
         <v>343</v>
       </c>
       <c r="E6" s="2" t="s">
@@ -5545,14 +5720,14 @@
         <v>441</v>
       </c>
     </row>
-    <row r="7" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="61" t="s">
         <v>360</v>
       </c>
       <c r="C7" s="60" t="s">
         <v>344</v>
       </c>
-      <c r="D7" s="76" t="s">
+      <c r="D7" s="70" t="s">
         <v>355</v>
       </c>
       <c r="E7" s="2"/>
@@ -5594,7 +5769,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="8" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
         <v>345</v>
@@ -5633,7 +5808,7 @@
       </c>
       <c r="T8" s="2"/>
     </row>
-    <row r="9" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="61"/>
       <c r="C9" s="57"/>
       <c r="D9" s="2" t="s">
@@ -5666,7 +5841,7 @@
       </c>
       <c r="T9" s="2"/>
     </row>
-    <row r="10" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="50"/>
       <c r="C10" s="57"/>
       <c r="D10" s="2" t="s">
@@ -5695,7 +5870,7 @@
       <c r="S10" s="2"/>
       <c r="T10" s="2"/>
     </row>
-    <row r="11" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="50"/>
       <c r="C11" s="57"/>
       <c r="D11" s="2"/>
@@ -5722,7 +5897,7 @@
       <c r="S11" s="61"/>
       <c r="T11" s="61"/>
     </row>
-    <row r="12" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="57"/>
       <c r="C12" s="57"/>
       <c r="D12" s="2"/>
@@ -5749,7 +5924,7 @@
       <c r="S12" s="61"/>
       <c r="T12" s="61"/>
     </row>
-    <row r="13" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="57"/>
       <c r="C13" s="57"/>
       <c r="D13" s="2"/>
@@ -5769,7 +5944,7 @@
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
     </row>
-    <row r="14" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="57"/>
       <c r="C14" s="57"/>
       <c r="D14" s="2"/>
@@ -5790,7 +5965,7 @@
       <c r="S14" s="2"/>
       <c r="T14" s="2"/>
     </row>
-    <row r="15" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="57"/>
       <c r="C15" s="57"/>
       <c r="D15" s="2"/>
@@ -5811,7 +5986,7 @@
       <c r="S15" s="2"/>
       <c r="T15" s="2"/>
     </row>
-    <row r="16" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="57"/>
       <c r="C16" s="57"/>
       <c r="D16" s="2"/>
@@ -5832,7 +6007,7 @@
       <c r="S16" s="2"/>
       <c r="T16" s="2"/>
     </row>
-    <row r="17" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="57"/>
       <c r="C17" s="57"/>
       <c r="D17" s="2"/>
@@ -5853,7 +6028,7 @@
       <c r="S17" s="2"/>
       <c r="T17" s="2"/>
     </row>
-    <row r="18" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="57"/>
       <c r="C18" s="57"/>
       <c r="D18" s="2"/>
@@ -5874,7 +6049,7 @@
       <c r="S18" s="2"/>
       <c r="T18" s="2"/>
     </row>
-    <row r="19" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="57"/>
       <c r="C19" s="57"/>
       <c r="D19" s="2"/>
@@ -5895,7 +6070,7 @@
       <c r="S19" s="2"/>
       <c r="T19" s="2"/>
     </row>
-    <row r="20" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="57"/>
       <c r="C20" s="57"/>
       <c r="D20" s="2"/>
@@ -5916,27 +6091,27 @@
       <c r="S20" s="2"/>
       <c r="T20" s="2"/>
     </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:20" x14ac:dyDescent="0.3">
       <c r="I21" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:20" x14ac:dyDescent="0.3">
       <c r="I22" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:20" x14ac:dyDescent="0.3">
       <c r="I23" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:20" x14ac:dyDescent="0.3">
       <c r="I24" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>327</v>
       </c>
@@ -5946,15 +6121,15 @@
       <c r="I25" s="19" t="s">
         <v>339</v>
       </c>
-      <c r="J25" s="70" t="s">
+      <c r="J25" s="72" t="s">
         <v>352</v>
       </c>
-      <c r="K25" s="70"/>
+      <c r="K25" s="72"/>
       <c r="N25" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>328</v>
       </c>
@@ -5977,7 +6152,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>329</v>
       </c>
@@ -6001,7 +6176,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>335</v>
       </c>
@@ -6022,7 +6197,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B29" s="20" t="s">
         <v>330</v>
       </c>
@@ -6039,7 +6214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:20" x14ac:dyDescent="0.3">
       <c r="F30" t="s">
         <v>364</v>
       </c>
@@ -6056,7 +6231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:20" x14ac:dyDescent="0.3">
       <c r="F31" s="19" t="s">
         <v>365</v>
       </c>
@@ -6076,7 +6251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:20" x14ac:dyDescent="0.3">
       <c r="F32" s="19">
         <v>1</v>
       </c>
@@ -6099,7 +6274,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B33" s="63" t="s">
         <v>400</v>
       </c>
@@ -6125,7 +6300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B34" s="63" t="s">
         <v>401</v>
       </c>
@@ -6157,7 +6332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B35" s="66">
         <v>1</v>
       </c>
@@ -6189,7 +6364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B36" s="66">
         <v>1</v>
       </c>
@@ -6212,7 +6387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B37" s="66">
         <v>1</v>
       </c>
@@ -6231,7 +6406,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B38" s="66">
         <v>2</v>
       </c>
@@ -6248,7 +6423,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B39" s="66">
         <v>2</v>
       </c>
@@ -6277,7 +6452,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B40" s="66">
         <v>2</v>
       </c>
@@ -6304,7 +6479,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B41" s="66">
         <v>2</v>
       </c>
@@ -6331,7 +6506,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B42" s="66"/>
       <c r="C42" s="66"/>
       <c r="D42" s="66"/>
@@ -6350,7 +6525,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B43" s="67"/>
       <c r="C43" s="67"/>
       <c r="D43" s="67"/>
@@ -6367,7 +6542,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B44" s="65"/>
       <c r="C44" s="65"/>
       <c r="D44" s="65"/>
@@ -6384,7 +6559,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.3">
       <c r="F45" s="19">
         <v>2</v>
       </c>
@@ -6397,7 +6572,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:11" x14ac:dyDescent="0.3">
       <c r="F46" s="19">
         <v>2</v>
       </c>
@@ -6410,7 +6585,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:11" x14ac:dyDescent="0.3">
       <c r="F47" s="19">
         <v>2</v>
       </c>
@@ -6423,42 +6598,42 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E49" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="50" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E50" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E51" t="s">
         <v>456</v>
       </c>
     </row>
-    <row r="53" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E53" t="s">
         <v>457</v>
       </c>
     </row>
-    <row r="54" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E54" t="s">
         <v>458</v>
       </c>
     </row>
-    <row r="56" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E56" t="s">
         <v>459</v>
       </c>
     </row>
-    <row r="57" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E57" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="58" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E58" t="s">
         <v>461</v>
       </c>
@@ -6480,17 +6655,373 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAA87FE5-CACE-4E39-9F24-2694403041B6}">
+  <dimension ref="B3:E35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="26.77734375" customWidth="1"/>
+    <col min="3" max="3" width="27.88671875" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" customWidth="1"/>
+    <col min="5" max="5" width="24.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B3" s="78" t="s">
+        <v>493</v>
+      </c>
+      <c r="C3" s="69"/>
+    </row>
+    <row r="4" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B4" s="79" t="s">
+        <v>494</v>
+      </c>
+      <c r="C4" s="80" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B5" s="25">
+        <v>1</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B6" s="25">
+        <v>2</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B7" s="25">
+        <v>3</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B8" s="25">
+        <v>4</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B9" s="25">
+        <v>5</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B10" s="25">
+        <v>6</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B11" s="25">
+        <v>7</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B14" s="78" t="s">
+        <v>332</v>
+      </c>
+      <c r="C14" s="69"/>
+      <c r="D14" s="69"/>
+    </row>
+    <row r="15" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B15" s="79" t="s">
+        <v>333</v>
+      </c>
+      <c r="C15" s="80" t="s">
+        <v>334</v>
+      </c>
+      <c r="D15" s="81" t="s">
+        <v>360</v>
+      </c>
+      <c r="E15" s="81" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B16" s="25">
+        <v>1</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>472</v>
+      </c>
+      <c r="D16" s="25">
+        <v>1</v>
+      </c>
+      <c r="E16" s="25"/>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B17" s="25">
+        <v>2</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>473</v>
+      </c>
+      <c r="D17" s="25">
+        <v>1</v>
+      </c>
+      <c r="E17" s="25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B18" s="25">
+        <v>3</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>474</v>
+      </c>
+      <c r="D18" s="25">
+        <v>1</v>
+      </c>
+      <c r="E18" s="25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B19" s="25">
+        <v>4</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>475</v>
+      </c>
+      <c r="D19" s="25">
+        <v>2</v>
+      </c>
+      <c r="E19" s="25"/>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B20" s="25">
+        <v>5</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>476</v>
+      </c>
+      <c r="D20" s="25">
+        <v>2</v>
+      </c>
+      <c r="E20" s="25"/>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B21" s="25">
+        <v>6</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>477</v>
+      </c>
+      <c r="D21" s="25">
+        <v>3</v>
+      </c>
+      <c r="E21" s="25"/>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B22" s="25">
+        <v>7</v>
+      </c>
+      <c r="C22" s="25" t="s">
+        <v>478</v>
+      </c>
+      <c r="D22" s="25">
+        <v>3</v>
+      </c>
+      <c r="E22" s="25"/>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B23" s="25">
+        <v>8</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>479</v>
+      </c>
+      <c r="D23" s="25">
+        <v>3</v>
+      </c>
+      <c r="E23" s="25"/>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B24" s="25">
+        <v>9</v>
+      </c>
+      <c r="C24" s="25" t="s">
+        <v>480</v>
+      </c>
+      <c r="D24" s="25">
+        <v>3</v>
+      </c>
+      <c r="E24" s="25"/>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B25" s="25">
+        <v>10</v>
+      </c>
+      <c r="C25" s="25" t="s">
+        <v>481</v>
+      </c>
+      <c r="D25" s="25">
+        <v>3</v>
+      </c>
+      <c r="E25" s="25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B26" s="25">
+        <v>11</v>
+      </c>
+      <c r="C26" s="25" t="s">
+        <v>482</v>
+      </c>
+      <c r="D26" s="25">
+        <v>4</v>
+      </c>
+      <c r="E26" s="25"/>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B27" s="25">
+        <v>12</v>
+      </c>
+      <c r="C27" s="25" t="s">
+        <v>483</v>
+      </c>
+      <c r="D27" s="25">
+        <v>1</v>
+      </c>
+      <c r="E27" s="25"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B28" s="25">
+        <v>13</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="D28" s="25">
+        <v>4</v>
+      </c>
+      <c r="E28" s="25"/>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B29" s="25">
+        <v>14</v>
+      </c>
+      <c r="C29" s="25" t="s">
+        <v>485</v>
+      </c>
+      <c r="D29" s="25">
+        <v>5</v>
+      </c>
+      <c r="E29" s="25"/>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B30" s="25">
+        <v>15</v>
+      </c>
+      <c r="C30" s="25" t="s">
+        <v>486</v>
+      </c>
+      <c r="D30" s="25">
+        <v>5</v>
+      </c>
+      <c r="E30" s="25"/>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B31" s="25">
+        <v>16</v>
+      </c>
+      <c r="C31" s="25" t="s">
+        <v>487</v>
+      </c>
+      <c r="D31" s="25">
+        <v>6</v>
+      </c>
+      <c r="E31" s="25"/>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B32" s="25">
+        <v>17</v>
+      </c>
+      <c r="C32" s="25" t="s">
+        <v>488</v>
+      </c>
+      <c r="D32" s="25">
+        <v>6</v>
+      </c>
+      <c r="E32" s="25"/>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B33" s="25">
+        <v>18</v>
+      </c>
+      <c r="C33" s="25" t="s">
+        <v>489</v>
+      </c>
+      <c r="D33" s="25">
+        <v>5</v>
+      </c>
+      <c r="E33" s="25"/>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B34" s="25">
+        <v>19</v>
+      </c>
+      <c r="C34" s="25" t="s">
+        <v>490</v>
+      </c>
+      <c r="D34" s="25">
+        <v>7</v>
+      </c>
+      <c r="E34" s="25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B35" s="25">
+        <v>20</v>
+      </c>
+      <c r="C35" s="25" t="s">
+        <v>491</v>
+      </c>
+      <c r="D35" s="25">
+        <v>7</v>
+      </c>
+      <c r="E35" s="25"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:AJ77"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="4" width="8.85546875" customWidth="1"/>
+    <col min="3" max="4" width="8.88671875" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="33" max="33" width="17.7109375" customWidth="1"/>
+    <col min="33" max="33" width="17.6640625" customWidth="1"/>
     <col min="34" max="34" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>76</v>
       </c>
@@ -6498,12 +7029,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="E3" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="E4" t="s">
         <v>79</v>
       </c>
@@ -6515,7 +7046,7 @@
       </c>
       <c r="U4" s="16"/>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
       <c r="E5" t="s">
         <v>80</v>
       </c>
@@ -6547,7 +7078,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
       <c r="E6" t="s">
         <v>81</v>
       </c>
@@ -6573,7 +7104,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>203</v>
       </c>
@@ -6599,7 +7130,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>75</v>
       </c>
@@ -6625,7 +7156,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>98</v>
       </c>
@@ -6642,7 +7173,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
       <c r="C10" s="19" t="s">
         <v>204</v>
       </c>
@@ -6672,7 +7203,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
         <v>205</v>
       </c>
@@ -6696,7 +7227,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
       <c r="P12" s="4" t="s">
         <v>67</v>
       </c>
@@ -6705,7 +7236,7 @@
       </c>
       <c r="R12" s="5"/>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
       <c r="P13" s="4" t="s">
         <v>85</v>
       </c>
@@ -6717,7 +7248,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
       <c r="B14" s="16" t="s">
         <v>0</v>
       </c>
@@ -6738,7 +7269,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
       <c r="B15" s="6" t="s">
         <v>1</v>
       </c>
@@ -6761,7 +7292,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
       <c r="B16" s="4" t="s">
         <v>22</v>
       </c>
@@ -6791,7 +7322,7 @@
       <c r="X16" s="9"/>
       <c r="Y16" s="9"/>
     </row>
-    <row r="17" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:35" x14ac:dyDescent="0.3">
       <c r="B17" s="4" t="s">
         <v>24</v>
       </c>
@@ -6811,7 +7342,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="18" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:35" x14ac:dyDescent="0.3">
       <c r="B18" s="4" t="s">
         <v>26</v>
       </c>
@@ -6837,7 +7368,7 @@
       <c r="V18" s="17"/>
       <c r="W18" s="5"/>
     </row>
-    <row r="19" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:35" x14ac:dyDescent="0.3">
       <c r="B19" s="4" t="s">
         <v>317</v>
       </c>
@@ -6850,10 +7381,10 @@
       <c r="E19" s="25" t="s">
         <v>321</v>
       </c>
-      <c r="P19" s="75" t="s">
+      <c r="P19" s="77" t="s">
         <v>11</v>
       </c>
-      <c r="Q19" s="75"/>
+      <c r="Q19" s="77"/>
       <c r="T19" s="4" t="s">
         <v>9</v>
       </c>
@@ -6867,14 +7398,14 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:35" x14ac:dyDescent="0.3">
       <c r="P20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="Q20" s="74" t="s">
+      <c r="Q20" s="76" t="s">
         <v>14</v>
       </c>
-      <c r="R20" s="74"/>
+      <c r="R20" s="76"/>
       <c r="T20" s="4" t="s">
         <v>94</v>
       </c>
@@ -6888,14 +7419,14 @@
         <v>67</v>
       </c>
     </row>
-    <row r="21" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:35" x14ac:dyDescent="0.3">
       <c r="P21" s="4">
         <v>1</v>
       </c>
-      <c r="Q21" s="74" t="s">
+      <c r="Q21" s="76" t="s">
         <v>99</v>
       </c>
-      <c r="R21" s="74"/>
+      <c r="R21" s="76"/>
       <c r="T21" s="4" t="s">
         <v>94</v>
       </c>
@@ -6909,17 +7440,17 @@
         <v>67</v>
       </c>
     </row>
-    <row r="22" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:35" x14ac:dyDescent="0.3">
       <c r="D22" t="s">
         <v>208</v>
       </c>
       <c r="P22" s="4">
         <v>2</v>
       </c>
-      <c r="Q22" s="74" t="s">
+      <c r="Q22" s="76" t="s">
         <v>100</v>
       </c>
-      <c r="R22" s="74"/>
+      <c r="R22" s="76"/>
       <c r="T22" s="4" t="s">
         <v>94</v>
       </c>
@@ -6933,7 +7464,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="23" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:35" x14ac:dyDescent="0.3">
       <c r="D23" s="22" t="s">
         <v>124</v>
       </c>
@@ -6943,10 +7474,10 @@
       <c r="P23" s="4">
         <v>3</v>
       </c>
-      <c r="Q23" s="74" t="s">
+      <c r="Q23" s="76" t="s">
         <v>101</v>
       </c>
-      <c r="R23" s="74"/>
+      <c r="R23" s="76"/>
       <c r="T23" s="4"/>
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
@@ -6961,7 +7492,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="24" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:35" x14ac:dyDescent="0.3">
       <c r="D24" s="4" t="s">
         <v>126</v>
       </c>
@@ -6973,10 +7504,10 @@
       <c r="P24" s="4">
         <v>4</v>
       </c>
-      <c r="Q24" s="74" t="s">
+      <c r="Q24" s="76" t="s">
         <v>102</v>
       </c>
-      <c r="R24" s="74"/>
+      <c r="R24" s="76"/>
       <c r="T24" s="4" t="s">
         <v>95</v>
       </c>
@@ -6996,7 +7527,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="25" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:35" x14ac:dyDescent="0.3">
       <c r="D25" s="4" t="s">
         <v>128</v>
       </c>
@@ -7009,7 +7540,7 @@
       <c r="L25" s="32"/>
       <c r="M25" s="30"/>
     </row>
-    <row r="26" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:35" x14ac:dyDescent="0.3">
       <c r="D26" s="4" t="s">
         <v>126</v>
       </c>
@@ -7017,7 +7548,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="27" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:35" x14ac:dyDescent="0.3">
       <c r="D27" s="8" t="s">
         <v>142</v>
       </c>
@@ -7025,7 +7556,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:35" x14ac:dyDescent="0.3">
       <c r="D28" s="4" t="s">
         <v>127</v>
       </c>
@@ -7047,7 +7578,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:35" x14ac:dyDescent="0.3">
       <c r="C29" s="17" t="s">
         <v>117</v>
       </c>
@@ -7097,7 +7628,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:35" x14ac:dyDescent="0.3">
       <c r="C30" s="6" t="s">
         <v>118</v>
       </c>
@@ -7165,7 +7696,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="31" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:35" x14ac:dyDescent="0.3">
       <c r="C31" s="43" t="s">
         <v>121</v>
       </c>
@@ -7233,7 +7764,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="32" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:35" x14ac:dyDescent="0.3">
       <c r="C32" s="43" t="s">
         <v>122</v>
       </c>
@@ -7301,7 +7832,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="33" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C33" s="43" t="s">
         <v>123</v>
       </c>
@@ -7363,7 +7894,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="34" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C34" s="43" t="s">
         <v>139</v>
       </c>
@@ -7395,7 +7926,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C35" s="43" t="s">
         <v>143</v>
       </c>
@@ -7418,7 +7949,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="37" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C37" s="29" t="s">
         <v>147</v>
       </c>
@@ -7453,7 +7984,7 @@
       <c r="AI37" s="9"/>
       <c r="AJ37" s="9"/>
     </row>
-    <row r="38" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C38" t="s">
         <v>133</v>
       </c>
@@ -7464,7 +7995,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="39" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C39" t="s">
         <v>134</v>
       </c>
@@ -7475,7 +8006,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="40" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C40" t="s">
         <v>213</v>
       </c>
@@ -7486,7 +8017,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="41" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C41" t="s">
         <v>132</v>
       </c>
@@ -7494,7 +8025,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="42" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C42" t="s">
         <v>135</v>
       </c>
@@ -7509,12 +8040,12 @@
       <c r="AG42" s="41"/>
       <c r="AH42" s="41"/>
     </row>
-    <row r="43" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C43" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="44" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C44" t="s">
         <v>141</v>
       </c>
@@ -7528,7 +8059,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="45" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C45" t="s">
         <v>137</v>
       </c>
@@ -7557,7 +8088,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="46" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C46" t="s">
         <v>138</v>
       </c>
@@ -7592,7 +8123,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="47" spans="3:36" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:36" x14ac:dyDescent="0.3">
       <c r="C47" t="s">
         <v>214</v>
       </c>
@@ -7624,17 +8155,17 @@
         <v>219</v>
       </c>
     </row>
-    <row r="48" spans="3:36" x14ac:dyDescent="0.25">
-      <c r="C48" s="71" t="s">
+    <row r="48" spans="3:36" x14ac:dyDescent="0.3">
+      <c r="C48" s="73" t="s">
         <v>216</v>
       </c>
-      <c r="D48" s="72"/>
-      <c r="E48" s="72"/>
-      <c r="F48" s="72"/>
-      <c r="G48" s="72"/>
-      <c r="H48" s="72"/>
-      <c r="I48" s="72"/>
-      <c r="J48" s="72"/>
+      <c r="D48" s="74"/>
+      <c r="E48" s="74"/>
+      <c r="F48" s="74"/>
+      <c r="G48" s="74"/>
+      <c r="H48" s="74"/>
+      <c r="I48" s="74"/>
+      <c r="J48" s="74"/>
       <c r="O48" s="25">
         <v>3</v>
       </c>
@@ -7663,17 +8194,17 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="3:32" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C49" s="73" t="s">
+    <row r="49" spans="3:32" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C49" s="75" t="s">
         <v>215</v>
       </c>
-      <c r="D49" s="73"/>
-      <c r="E49" s="73"/>
-      <c r="F49" s="73"/>
-      <c r="G49" s="73"/>
-      <c r="H49" s="73"/>
-      <c r="I49" s="73"/>
-      <c r="J49" s="73"/>
+      <c r="D49" s="75"/>
+      <c r="E49" s="75"/>
+      <c r="F49" s="75"/>
+      <c r="G49" s="75"/>
+      <c r="H49" s="75"/>
+      <c r="I49" s="75"/>
+      <c r="J49" s="75"/>
       <c r="O49" s="25">
         <v>4</v>
       </c>
@@ -7702,7 +8233,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="50" spans="3:32" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:32" x14ac:dyDescent="0.3">
       <c r="O50" s="25">
         <v>5</v>
       </c>
@@ -7722,7 +8253,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="51" spans="3:32" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:32" x14ac:dyDescent="0.3">
       <c r="O51" s="25">
         <v>6</v>
       </c>
@@ -7742,7 +8273,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="52" spans="3:32" x14ac:dyDescent="0.25">
+    <row r="52" spans="3:32" x14ac:dyDescent="0.3">
       <c r="C52" s="17" t="s">
         <v>117</v>
       </c>
@@ -7768,7 +8299,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="53" spans="3:32" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:32" x14ac:dyDescent="0.3">
       <c r="C53" s="6" t="s">
         <v>118</v>
       </c>
@@ -7803,7 +8334,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="54" spans="3:32" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:32" x14ac:dyDescent="0.3">
       <c r="C54" s="43" t="s">
         <v>121</v>
       </c>
@@ -7831,7 +8362,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="55" spans="3:32" x14ac:dyDescent="0.25">
+    <row r="55" spans="3:32" x14ac:dyDescent="0.3">
       <c r="C55" s="43" t="s">
         <v>122</v>
       </c>
@@ -7869,7 +8400,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="56" spans="3:32" x14ac:dyDescent="0.25">
+    <row r="56" spans="3:32" x14ac:dyDescent="0.3">
       <c r="C56" s="43" t="s">
         <v>123</v>
       </c>
@@ -7904,7 +8435,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="57" spans="3:32" x14ac:dyDescent="0.25">
+    <row r="57" spans="3:32" x14ac:dyDescent="0.3">
       <c r="C57" s="43" t="s">
         <v>139</v>
       </c>
@@ -7930,7 +8461,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="58" spans="3:32" x14ac:dyDescent="0.25">
+    <row r="58" spans="3:32" x14ac:dyDescent="0.3">
       <c r="C58" s="43" t="s">
         <v>143</v>
       </c>
@@ -7956,7 +8487,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="59" spans="3:32" x14ac:dyDescent="0.25">
+    <row r="59" spans="3:32" x14ac:dyDescent="0.3">
       <c r="O59" s="25">
         <v>14</v>
       </c>
@@ -7970,7 +8501,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="60" spans="3:32" x14ac:dyDescent="0.25">
+    <row r="60" spans="3:32" x14ac:dyDescent="0.3">
       <c r="O60" s="25">
         <v>15</v>
       </c>
@@ -7984,7 +8515,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="61" spans="3:32" x14ac:dyDescent="0.25">
+    <row r="61" spans="3:32" x14ac:dyDescent="0.3">
       <c r="O61" s="25">
         <v>16</v>
       </c>
@@ -7998,7 +8529,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="71" spans="17:24" x14ac:dyDescent="0.25">
+    <row r="71" spans="17:24" x14ac:dyDescent="0.3">
       <c r="Q71" s="17" t="s">
         <v>117</v>
       </c>
@@ -8007,7 +8538,7 @@
       </c>
       <c r="X71" s="18"/>
     </row>
-    <row r="72" spans="17:24" x14ac:dyDescent="0.25">
+    <row r="72" spans="17:24" x14ac:dyDescent="0.3">
       <c r="Q72" s="6" t="s">
         <v>118</v>
       </c>
@@ -8027,7 +8558,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="73" spans="17:24" x14ac:dyDescent="0.25">
+    <row r="73" spans="17:24" x14ac:dyDescent="0.3">
       <c r="Q73" s="4" t="s">
         <v>121</v>
       </c>
@@ -8047,7 +8578,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="74" spans="17:24" x14ac:dyDescent="0.25">
+    <row r="74" spans="17:24" x14ac:dyDescent="0.3">
       <c r="Q74" s="4" t="s">
         <v>122</v>
       </c>
@@ -8067,7 +8598,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="75" spans="17:24" x14ac:dyDescent="0.25">
+    <row r="75" spans="17:24" x14ac:dyDescent="0.3">
       <c r="Q75" s="4" t="s">
         <v>123</v>
       </c>
@@ -8087,7 +8618,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="76" spans="17:24" x14ac:dyDescent="0.25">
+    <row r="76" spans="17:24" x14ac:dyDescent="0.3">
       <c r="Q76" s="4" t="s">
         <v>139</v>
       </c>
@@ -8101,7 +8632,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="77" spans="17:24" x14ac:dyDescent="0.25">
+    <row r="77" spans="17:24" x14ac:dyDescent="0.3">
       <c r="Q77" s="4" t="s">
         <v>143</v>
       </c>

</xml_diff>